<commit_message>
Setup Google Auth infrastructure and base quiz logic
</commit_message>
<xml_diff>
--- a/question.xlsx
+++ b/question.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\חני\תשפו\JAVA\שלי\project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\חני\תשפו\JAVA\שלי\project\QuizPlatform\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E45562F-75F5-4B91-BDBD-A4561985C682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A469D71F-9A1B-46C7-B324-CC7F4C58BDCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="46">
   <si>
     <t>2+2</t>
   </si>
@@ -52,6 +52,117 @@
   </si>
   <si>
     <t>??</t>
+  </si>
+  <si>
+    <t>מהי בירת צרפת?</t>
+  </si>
+  <si>
+    <t>פריז</t>
+  </si>
+  <si>
+    <t>ברלין</t>
+  </si>
+  <si>
+    <t>רומא</t>
+  </si>
+  <si>
+    <t>מדריד</t>
+  </si>
+  <si>
+    <t>כמה ימים יש בשנה רגילה?</t>
+  </si>
+  <si>
+    <t>איזה כוכב הוא הקרוב ביותר לשמש?</t>
+  </si>
+  <si>
+    <t>חמה</t>
+  </si>
+  <si>
+    <t>נוגה</t>
+  </si>
+  <si>
+    <t>צדק</t>
+  </si>
+  <si>
+    <t>מאדים</t>
+  </si>
+  <si>
+    <t>כמה מיתרים יש לגיטרה רגילה?</t>
+  </si>
+  <si>
+    <t>איזה כלי נגינה שייך למשפחת כלי הנשיפה?</t>
+  </si>
+  <si>
+    <t>חליל</t>
+  </si>
+  <si>
+    <t>חליל צד</t>
+  </si>
+  <si>
+    <t>כינור</t>
+  </si>
+  <si>
+    <t>תוף</t>
+  </si>
+  <si>
+    <t>פסנתר</t>
+  </si>
+  <si>
+    <t>מה שוקל יותר?</t>
+  </si>
+  <si>
+    <t>שניהם אותו דבר</t>
+  </si>
+  <si>
+    <t>תלוי בגודל</t>
+  </si>
+  <si>
+    <t>קילו נוצות</t>
+  </si>
+  <si>
+    <t>קילו ברזל</t>
+  </si>
+  <si>
+    <t>איזה כלי נגינה כולל קלידים ומיתרים?</t>
+  </si>
+  <si>
+    <t>חצוצרה</t>
+  </si>
+  <si>
+    <t>איזה כלי נגינה מנגנים בעזרת קשת?</t>
+  </si>
+  <si>
+    <t>גיטרה</t>
+  </si>
+  <si>
+    <t>כמה קלידים יש בדרך כלל בפסנתר מלא?</t>
+  </si>
+  <si>
+    <t>איזה כלי נגינה הוא הגדול ביותר במשפחת כלי הקשת?</t>
+  </si>
+  <si>
+    <t>קונטרבס</t>
+  </si>
+  <si>
+    <t>צ'לו</t>
+  </si>
+  <si>
+    <t>ויולה</t>
+  </si>
+  <si>
+    <t>איזה כלי נגינה משתמשים בו לעיתים קרובות בג'אז?</t>
+  </si>
+  <si>
+    <t>סקסופון</t>
+  </si>
+  <si>
+    <t>נבל</t>
+  </si>
+  <si>
+    <t>קסילופון</t>
+  </si>
+  <si>
+    <t>טובה</t>
   </si>
 </sst>
 </file>
@@ -87,8 +198,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -369,7 +483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -432,6 +546,226 @@
         <v>10</v>
       </c>
     </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5">
+        <v>365</v>
+      </c>
+      <c r="C5">
+        <v>366</v>
+      </c>
+      <c r="D5">
+        <v>355</v>
+      </c>
+      <c r="E5">
+        <v>360</v>
+      </c>
+      <c r="F5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>7</v>
+      </c>
+      <c r="F7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12">
+        <v>88</v>
+      </c>
+      <c r="C12">
+        <v>100</v>
+      </c>
+      <c r="D12">
+        <v>66</v>
+      </c>
+      <c r="E12">
+        <v>72</v>
+      </c>
+      <c r="F12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" t="s">
+        <v>45</v>
+      </c>
+      <c r="F14">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Final push - core functionality complete (minor tweaks pending)
</commit_message>
<xml_diff>
--- a/question.xlsx
+++ b/question.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\חני\תשפו\JAVA\שלי\project\QuizPlatform\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A469D71F-9A1B-46C7-B324-CC7F4C58BDCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEDD2450-4969-4020-AB03-002851E1BB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -108,9 +108,6 @@
     <t>פסנתר</t>
   </si>
   <si>
-    <t>מה שוקל יותר?</t>
-  </si>
-  <si>
     <t>שניהם אותו דבר</t>
   </si>
   <si>
@@ -129,9 +126,6 @@
     <t>חצוצרה</t>
   </si>
   <si>
-    <t>איזה כלי נגינה מנגנים בעזרת קשת?</t>
-  </si>
-  <si>
     <t>גיטרה</t>
   </si>
   <si>
@@ -163,6 +157,12 @@
   </si>
   <si>
     <t>טובה</t>
+  </si>
+  <si>
+    <t>מה שוקל יותר? קילו ברזל או קילו נוצות?</t>
+  </si>
+  <si>
+    <t>באיזה כלי נגינה מנגנים בעזרת קשת?</t>
   </si>
 </sst>
 </file>
@@ -648,19 +648,19 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" t="s">
         <v>27</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" t="s">
         <v>29</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>30</v>
-      </c>
-      <c r="E9" t="s">
-        <v>31</v>
       </c>
       <c r="F9">
         <v>5</v>
@@ -668,13 +668,13 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
         <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D10" t="s">
         <v>22</v>
@@ -688,13 +688,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="B11" t="s">
         <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D11" t="s">
         <v>22</v>
@@ -708,7 +708,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B12">
         <v>88</v>
@@ -728,16 +728,16 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" t="s">
         <v>37</v>
       </c>
-      <c r="B13" t="s">
+      <c r="D13" t="s">
         <v>38</v>
-      </c>
-      <c r="C13" t="s">
-        <v>39</v>
-      </c>
-      <c r="D13" t="s">
-        <v>40</v>
       </c>
       <c r="E13" t="s">
         <v>24</v>
@@ -748,19 +748,19 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" t="s">
         <v>41</v>
       </c>
-      <c r="B14" t="s">
+      <c r="D14" t="s">
         <v>42</v>
       </c>
-      <c r="C14" t="s">
+      <c r="E14" t="s">
         <v>43</v>
-      </c>
-      <c r="D14" t="s">
-        <v>44</v>
-      </c>
-      <c r="E14" t="s">
-        <v>45</v>
       </c>
       <c r="F14">
         <v>10</v>

</xml_diff>

<commit_message>
Commit before uploading to render
</commit_message>
<xml_diff>
--- a/question.xlsx
+++ b/question.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\חני\תשפו\JAVA\שלי\project\QuizPlatform\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEDD2450-4969-4020-AB03-002851E1BB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569D7B9D-08FE-4BE1-8ABF-12DC0C9364E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,9 +51,6 @@
     <t>אהרלה סמט</t>
   </si>
   <si>
-    <t>??</t>
-  </si>
-  <si>
     <t>מהי בירת צרפת?</t>
   </si>
   <si>
@@ -163,6 +160,9 @@
   </si>
   <si>
     <t>באיזה כלי נגינה מנגנים בעזרת קשת?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">שוכי גולדשטיין </t>
   </si>
 </sst>
 </file>
@@ -198,11 +198,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -539,8 +540,8 @@
       <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" t="s">
-        <v>8</v>
+      <c r="E3" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="F3">
         <v>10</v>
@@ -548,19 +549,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>12</v>
-      </c>
-      <c r="E4" t="s">
-        <v>13</v>
       </c>
       <c r="F4">
         <v>10</v>
@@ -568,7 +569,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5">
         <v>365</v>
@@ -588,19 +589,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
         <v>15</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>16</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>17</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>18</v>
-      </c>
-      <c r="E6" t="s">
-        <v>19</v>
       </c>
       <c r="F6">
         <v>10</v>
@@ -608,7 +609,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7">
         <v>6</v>
@@ -628,19 +629,19 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
         <v>23</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>24</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>25</v>
-      </c>
-      <c r="E8" t="s">
-        <v>26</v>
       </c>
       <c r="F8">
         <v>5</v>
@@ -648,19 +649,19 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" t="s">
         <v>28</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>29</v>
-      </c>
-      <c r="E9" t="s">
-        <v>30</v>
       </c>
       <c r="F9">
         <v>5</v>
@@ -668,19 +669,19 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
         <v>31</v>
       </c>
-      <c r="B10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" t="s">
-        <v>32</v>
-      </c>
       <c r="D10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F10">
         <v>10</v>
@@ -688,19 +689,19 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" t="s">
         <v>24</v>
-      </c>
-      <c r="C11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" t="s">
-        <v>25</v>
       </c>
       <c r="F11">
         <v>5</v>
@@ -708,7 +709,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B12">
         <v>88</v>
@@ -728,19 +729,19 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" t="s">
         <v>35</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>36</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>37</v>
       </c>
-      <c r="D13" t="s">
-        <v>38</v>
-      </c>
       <c r="E13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F13">
         <v>5</v>
@@ -748,19 +749,19 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
         <v>39</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>40</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>41</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>42</v>
-      </c>
-      <c r="E14" t="s">
-        <v>43</v>
       </c>
       <c r="F14">
         <v>10</v>
@@ -768,5 +769,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>